<commit_message>
Updated HowTo sheets for connections, types, and groups
</commit_message>
<xml_diff>
--- a/public/exportTemplates/connections.xlsx
+++ b/public/exportTemplates/connections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TempShare\KYVL_CC_Plus\Export samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38064827-3D51-41C0-A12F-2F584DEF581C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F72DDB1-455D-42D7-BBAC-C7ADE26EEC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="4110" windowWidth="24645" windowHeight="14385" xr2:uid="{D5135CBE-1346-4875-9AA3-E4BF32C48D4E}"/>
+    <workbookView xWindow="285" yWindow="4335" windowWidth="19590" windowHeight="15795" xr2:uid="{D5135CBE-1346-4875-9AA3-E4BF32C48D4E}"/>
   </bookViews>
   <sheets>
     <sheet name="HowToImport" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
   <si>
     <t>Column Name</t>
   </si>
@@ -69,102 +69,54 @@
     <t xml:space="preserve"> * Once the data sheet contains everything to be updated or inserted, save the sheet as a CSV UTF-8 file and import it into CC-Plus.</t>
   </si>
   <si>
-    <t xml:space="preserve"> * The Connections tab represents a starting place for updating or importing settings.</t>
-  </si>
-  <si>
-    <t>Connection imports cannot be used to delete existing connections; only additions and updates are supported.</t>
-  </si>
-  <si>
     <t>Platform Name</t>
   </si>
   <si>
     <t>String</t>
   </si>
   <si>
-    <t>PR is ConsoWide</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>Y or N : Determines if  PR reports should be available consortium-wide</t>
-  </si>
-  <si>
     <t>PR Inst ID(s)</t>
   </si>
   <si>
     <t>CSV list</t>
   </si>
   <si>
-    <t>Institution IDs connected for PR reports</t>
-  </si>
-  <si>
     <t>PR Group ID(s)</t>
   </si>
   <si>
     <t>InstitutionGroup IDs connected for PR reports</t>
   </si>
   <si>
-    <t>DR is ConsoWide</t>
-  </si>
-  <si>
     <t>DR Inst ID(s)</t>
   </si>
   <si>
     <t>DR Group ID(s)</t>
   </si>
   <si>
-    <t>Y or N : Determines if  DR reports should be available consortium-wide</t>
-  </si>
-  <si>
-    <t>Institution IDs connected for DR reports</t>
-  </si>
-  <si>
     <t>InstitutionGroup IDs connected for DR reports</t>
   </si>
   <si>
-    <t>TR is ConsoWide</t>
-  </si>
-  <si>
     <t>TR Inst ID(s)</t>
   </si>
   <si>
     <t>TR Group ID(s)</t>
   </si>
   <si>
-    <t>Y or N : Determines if  TR reports should be available consortium-wide</t>
-  </si>
-  <si>
-    <t>Institution IDs connected for TR reports</t>
-  </si>
-  <si>
     <t>InstitutionGroup IDs connected for TR reports</t>
   </si>
   <si>
-    <t>IR is ConsoWide</t>
-  </si>
-  <si>
     <t>IR Inst ID(s)</t>
   </si>
   <si>
     <t>IR Group ID(s)</t>
   </si>
   <si>
-    <t>Y or N : Determines if  IR reports should be available consortium-wide</t>
-  </si>
-  <si>
-    <t>Institution IDs connected for IR reports</t>
-  </si>
-  <si>
     <t>InstitutionGroup IDs connected for IR reports</t>
   </si>
   <si>
     <t xml:space="preserve"> * The header row and all columns beyond 'N' will be ignored.</t>
   </si>
   <si>
-    <t xml:space="preserve"> * If values are missing or invalid for columns (C-N), but not required, they will be set to the 'Default'.</t>
-  </si>
-  <si>
     <t>Platform Name (included for readability only); NOT Imported</t>
   </si>
   <si>
@@ -175,13 +127,49 @@
   </si>
   <si>
     <t>* The safest approach is to update an existing full export to  avoid overwriting or deleting existing connections.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> * Including institution ID:1 in any of the "Inst ID(s)" columns (C,E,G, or I) will establish consortium-wide connection(s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    (In this case, any other Institution ID(s) or Group ID(s) supplied for the Platform will be redundant, and ignored.)</t>
+  </si>
+  <si>
+    <t>Institution IDs connected for PR reports (including  1 sets conso-wide)</t>
+  </si>
+  <si>
+    <t>Institution IDs connected for DR reports (including  1  sets conso-wide)</t>
+  </si>
+  <si>
+    <t>Institution IDs connected for TR reports (including  1  sets conso-wide)</t>
+  </si>
+  <si>
+    <t>Institution IDs connected for IR reports (including  1  sets conso-wide)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> * If a report (PR, TR, etc.) is not available for the platform for column-A, the Inst and Group ID(s) for that report are ignored</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> * If values are missing or invalid for columns (C-J), but not required, they will be set to the 'Default'.</t>
+  </si>
+  <si>
+    <t>( removing/omitting and institution or group from the sets of IDs removes the report-mapping. If all report mappings are removed/missing,</t>
+  </si>
+  <si>
+    <t>for a given institution/group, the internal, parent connection record will also be removed)</t>
+  </si>
+  <si>
+    <t>Connection imports function as FULL REPLACEMENT of rows given as input, and will ADD , UPDATE, or REMOVE connection assignments!</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> * The Connections tab represents a starting place for updating or importing settings, and will act as a FULL REPLACEMENT for platforms given as input!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -207,6 +195,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -308,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -332,6 +325,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -636,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64B1D0BC-6658-4CFF-BA97-66628E7E0E3E}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
@@ -655,7 +650,7 @@
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
@@ -664,7 +659,7 @@
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -673,7 +668,7 @@
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -691,7 +686,7 @@
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -699,15 +694,17 @@
       <c r="E6" s="10"/>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
+      <c r="A7" s="8" t="s">
+        <v>34</v>
+      </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="10"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>12</v>
+      <c r="A8" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -715,156 +712,114 @@
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="10"/>
+    </row>
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="10"/>
+    </row>
+    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="13"/>
-    </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4"/>
-      <c r="B10" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18"/>
-    </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="B12" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="13"/>
+    </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="20"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="B14" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="20"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="18"/>
+    </row>
+    <row r="16" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" spans="1:5" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>19</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>30</v>
@@ -873,18 +828,18 @@
         <v>9</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>9</v>
@@ -895,30 +850,30 @@
     </row>
     <row r="22" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>9</v>
@@ -929,13 +884,13 @@
     </row>
     <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>9</v>
@@ -946,30 +901,30 @@
     </row>
     <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>9</v>
@@ -980,13 +935,13 @@
     </row>
     <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>9</v>
@@ -995,27 +950,49 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="11">
+  <mergeCells count="16">
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A10:E10"/>
     <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B12:E12"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
-    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>